<commit_message>
working on react exercises
</commit_message>
<xml_diff>
--- a/DN - Java FSE Mandatory hands-on detail (1).xlsx
+++ b/DN - Java FSE Mandatory hands-on detail (1).xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="96">
   <si>
     <t>Skill</t>
   </si>
@@ -314,6 +314,15 @@
   </si>
   <si>
     <t>Angular Hands-on</t>
+  </si>
+  <si>
+    <t>https://github.com/Naresh-Chaurasia/GenC-React</t>
+  </si>
+  <si>
+    <t>https://github.com/Naresh-Chaurasia/GenC-KnowledgeHub/blob/main/gen-c/javascript/genc-javascript.adoc</t>
+  </si>
+  <si>
+    <t>https://github.com/Naresh-Chaurasia/GenC-KnowledgeHub</t>
   </si>
 </sst>
 </file>
@@ -838,7 +847,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23.125" customWidth="1"/>
@@ -1519,6 +1528,21 @@
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8"/>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" t="s">
+        <v>95</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>